<commit_message>
Publish Duisburg_2012_WC, London_2012_OG, Moscow_2012_WC, Poznan_2012_WC, Rome_2012_MAR
</commit_message>
<xml_diff>
--- a/events/Duisburg_2012_WC/Duisburg_2012_WC_Results.xlsx
+++ b/events/Duisburg_2012_WC/Duisburg_2012_WC_Results.xlsx
@@ -7522,6 +7522,11 @@
           <t>00:04:49.661</t>
         </is>
       </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -25548,6 +25553,11 @@
           <t>00:02:09.882</t>
         </is>
       </c>
+      <c r="R393" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -32480,6 +32490,11 @@
           <t>00:02:14.763</t>
         </is>
       </c>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -50291,6 +50306,11 @@
           <t>00:00:46.235</t>
         </is>
       </c>
+      <c r="R769" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr">
@@ -63914,6 +63934,11 @@
           <t>00:00:46.028</t>
         </is>
       </c>
+      <c r="R981" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
     </row>
     <row r="982">
       <c r="A982" t="inlineStr">
@@ -82835,6 +82860,11 @@
       <c r="P1270" t="inlineStr">
         <is>
           <t>00:02:07.331</t>
+        </is>
+      </c>
+      <c r="R1270" t="inlineStr">
+        <is>
+          <t>51939</t>
         </is>
       </c>
     </row>
@@ -89456,7 +89486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D272"/>
+  <dimension ref="A1:D273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95443,6 +95473,28 @@
         </is>
       </c>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>51939</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Vicente</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Gonzales</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>